<commit_message>
Carga masiva: Origen pasa a texto libre (país de procedencia)
La columna Origen ya no valida contra solo "local"/"importado" — es
texto libre para indicar de qué país viene el producto (Guatemala,
China, Estados Unidos...). Origen no afecta el cálculo de precio desde
que el margen depende del nivel de ganancia, así que este cambio es
puramente descriptivo. Se ajusta la inferencia del tipo de proveedor
autocreado (local/importado sigue siendo binario, solo se infiere del
texto de origen en vez de copiarlo literal). El resto de los flujos
(alta manual, compras) no cambia — ya escriben valores de texto
válidos ("local"/"importado") bajo la nueva validación más permisiva.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantillas/articulos.xlsx
+++ b/public/plantillas/articulos.xlsx
@@ -100,7 +100,7 @@
     <t>Importación</t>
   </si>
   <si>
-    <t>local</t>
+    <t>Guatemala</t>
   </si>
   <si>
     <t>Oro</t>
@@ -172,7 +172,7 @@
     <t>Socio Comercial</t>
   </si>
   <si>
-    <t>importado</t>
+    <t>China</t>
   </si>
   <si>
     <t>novedad</t>

</xml_diff>

<commit_message>
Carga masiva: costo por gramo y eliminar borradores subidos por error
1) Cuando la fila trae "Peso (gramos)", "Coste" se interpreta como
   costo por gramo — el costo real de la pieza es Coste × Peso. Sin
   peso, Coste sigue siendo el costo total como hasta ahora. Se agrega
   columna "Costo total" en la previsualización para verificar el
   cálculo antes de confirmar la carga.

2) Nuevo botón "Eliminar" en Producción para borradores (en_produccion)
   — soft-delete (activo=false) vía fn_eliminar_producto_borrador, con
   confirmación antes de enviar. Solo aplica a piezas sin publicar:
   una vez en el CEDI, la corrección correcta es darla de baja, no
   eliminarla. Producción solo puede eliminar lo que ella misma creó;
   admin puede eliminar cualquier borrador.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantillas/articulos.xlsx
+++ b/public/plantillas/articulos.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="56">
   <si>
     <t>Referencia Interna (código)</t>
   </si>
@@ -112,7 +112,7 @@
     <t>novedad,edición limitada</t>
   </si>
   <si>
-    <t>Anillo clásico de compromiso — pieza única, se sube con Cantidad 1</t>
+    <t>Anillo clásico de compromiso — pieza única, se sube con Cantidad 1. Coste es por gramo (450/g × 3.25g = 1462.50 total)</t>
   </si>
   <si>
     <t>14k</t>
@@ -142,7 +142,7 @@
     <t>Primavera</t>
   </si>
   <si>
-    <t>Conjunto de algodón, corte holgado</t>
+    <t>Conjunto de algodón, corte holgado — sin peso, Coste es el costo total (60)</t>
   </si>
   <si>
     <t>M</t>
@@ -178,7 +178,7 @@
     <t>novedad</t>
   </si>
   <si>
-    <t>Audífonos bluetooth con estuche de carga</t>
+    <t>Audífonos bluetooth con estuche de carga — sin peso, Coste es el costo total (250)</t>
   </si>
 </sst>
 </file>
@@ -652,7 +652,7 @@
         <v>23</v>
       </c>
       <c r="B2">
-        <v>1500</v>
+        <v>450</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -802,8 +802,8 @@
       <c r="D4" t="s">
         <v>48</v>
       </c>
-      <c r="E4">
-        <v>0.35</v>
+      <c r="E4" t="s">
+        <v>24</v>
       </c>
       <c r="F4" t="s">
         <v>49</v>

</xml_diff>